<commit_message>
feat: add navigation tests
</commit_message>
<xml_diff>
--- a/docs/test-cases/TestCases_1.0.xlsx
+++ b/docs/test-cases/TestCases_1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORK\LEARNING\QA Engineer\Internship\5t-wdio-telnyx\docs\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67C98C7E-C2B5-453F-A265-FED93FC91677}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4292FE4F-918B-4393-BA99-74431C7DDFEC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -111,9 +111,6 @@
     <t>Verify Login form validation using an invalid email format</t>
   </si>
   <si>
-    <t>Verify the Solutions mega menu displays the expected navigation sections and primary options</t>
-  </si>
-  <si>
     <t>The login page was opened</t>
   </si>
   <si>
@@ -4066,6 +4063,9 @@
       </rPr>
       <t xml:space="preserve"> page was opened</t>
     </r>
+  </si>
+  <si>
+    <t>Verify the Solutions mega menu displays the primary solution cards and navigation links</t>
   </si>
 </sst>
 </file>
@@ -4484,10 +4484,10 @@
         <v>10</v>
       </c>
       <c r="D2" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>32</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>33</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>6</v>
@@ -4505,10 +4505,10 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>34</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>35</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>6</v>
@@ -4520,16 +4520,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>28</v>
+        <v>73</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>37</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>7</v>
@@ -4547,10 +4547,10 @@
         <v>11</v>
       </c>
       <c r="D5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>7</v>
@@ -4568,10 +4568,10 @@
         <v>11</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>40</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>41</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>6</v>
@@ -4586,13 +4586,13 @@
         <v>27</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D7" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>42</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>43</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>6</v>
@@ -4610,10 +4610,10 @@
         <v>11</v>
       </c>
       <c r="D8" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>45</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>6</v>
@@ -4628,13 +4628,13 @@
         <v>9</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D9" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>46</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>47</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>6</v>
@@ -4652,10 +4652,10 @@
         <v>11</v>
       </c>
       <c r="D10" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>48</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>49</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>6</v>
@@ -4673,10 +4673,10 @@
         <v>10</v>
       </c>
       <c r="D11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>50</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>51</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>7</v>
@@ -4691,13 +4691,13 @@
         <v>24</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D12" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>52</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>53</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>7</v>
@@ -4715,10 +4715,10 @@
         <v>11</v>
       </c>
       <c r="D13" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>54</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>55</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>7</v>
@@ -4733,13 +4733,13 @@
         <v>22</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D14" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>69</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>70</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>6</v>
@@ -4757,10 +4757,10 @@
         <v>11</v>
       </c>
       <c r="D15" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" s="5" t="s">
         <v>57</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>58</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>7</v>
@@ -4778,10 +4778,10 @@
         <v>11</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>7</v>
@@ -4793,16 +4793,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D17" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E17" s="5" t="s">
         <v>72</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>73</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>7</v>
@@ -4820,10 +4820,10 @@
         <v>11</v>
       </c>
       <c r="D18" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E18" s="5" t="s">
         <v>61</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>62</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>7</v>
@@ -4841,10 +4841,10 @@
         <v>10</v>
       </c>
       <c r="D19" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E19" s="5" t="s">
         <v>63</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>64</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>7</v>
@@ -4861,10 +4861,10 @@
         <v>11</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>7</v>
@@ -4882,10 +4882,10 @@
         <v>11</v>
       </c>
       <c r="D21" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="E21" s="5" t="s">
         <v>67</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>68</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
feat: add login validation tests
</commit_message>
<xml_diff>
--- a/docs/test-cases/TestCases_1.0.xlsx
+++ b/docs/test-cases/TestCases_1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORK\LEARNING\QA Engineer\Internship\5t-wdio-telnyx\docs\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4292FE4F-918B-4393-BA99-74431C7DDFEC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89448413-5C61-40A1-A04C-94D7617FCF73}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1068,268 +1068,6 @@
         <charset val="204"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Log In</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> header button is visible and enabled
-2. Click the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Log In</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> button
-3. Click the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Sign In With Password
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">4. Verify the email and password fields are empty.
-5. Click the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Log In</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> button</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. The </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Log In</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> header button was visible and enabled
-2. The login page was opened
-3. The email and password fields were displayed
-4. The email and password fields were empty
-5. The browser validation for the required email field was displayed</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. Verify the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Email</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> field is displayed
-2. Enter an invalid email address into the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Email</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> field
-3. Click the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Send me sign-in link</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> button</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. The </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Email</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> field was displayed
-2. The </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Email</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> field was populated with invalid email address
-3. The validation message for invalid email address was displayed</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. Verify the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>Pricing</t>
     </r>
     <r>
@@ -4066,6 +3804,245 @@
   </si>
   <si>
     <t>Verify the Solutions mega menu displays the primary solution cards and navigation links</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Verify the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Log In</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> header button is visible and enabled
+2. Click the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Log In</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> button
+3. Click the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Sign In With Password
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4. Verify the email and password fields are empty.
+5. Fill the required fields with invalid data</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Log In</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> header button was visible and enabled
+2. The login page was opened
+3. The email and password fields were displayed
+4. The email and password fields were empty
+5. The validation message for invalid email address was displayed</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Verify the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Email</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> field is displayed
+2. Verify the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Email</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> field is empty.
+3. Click the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Send me sign-in link</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> button</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Email</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> field was displayed
+2. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Email</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> field was empty
+3. The error notification with the message "Email is required" was displayed</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -4520,7 +4497,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>11</v>
@@ -4562,16 +4539,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>40</v>
+        <v>71</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>6</v>
@@ -4583,16 +4560,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>28</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>6</v>
@@ -4610,10 +4587,10 @@
         <v>11</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>6</v>
@@ -4631,10 +4608,10 @@
         <v>29</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>6</v>
@@ -4652,10 +4629,10 @@
         <v>11</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>6</v>
@@ -4673,10 +4650,10 @@
         <v>10</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>7</v>
@@ -4694,10 +4671,10 @@
         <v>30</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>7</v>
@@ -4715,10 +4692,10 @@
         <v>11</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>7</v>
@@ -4733,13 +4710,13 @@
         <v>22</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>6</v>
@@ -4757,10 +4734,10 @@
         <v>11</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>7</v>
@@ -4778,10 +4755,10 @@
         <v>11</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>7</v>
@@ -4793,16 +4770,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>7</v>
@@ -4820,10 +4797,10 @@
         <v>11</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>7</v>
@@ -4841,10 +4818,10 @@
         <v>10</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>7</v>
@@ -4861,10 +4838,10 @@
         <v>11</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>7</v>
@@ -4882,10 +4859,10 @@
         <v>11</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
feat: add ui tests
</commit_message>
<xml_diff>
--- a/docs/test-cases/TestCases_1.0.xlsx
+++ b/docs/test-cases/TestCases_1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORK\LEARNING\QA Engineer\Internship\5t-wdio-telnyx\docs\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5D51BEA-E672-4E31-8870-15096C1FE8FB}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D361D3A-DF76-456B-B8B6-E5B817299178}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1906,235 +1906,6 @@
 6. The cookie banner was not displayed</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">1. Verify the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Developer</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> menu is visible and enabled
-2. Click the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Developer</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> menu
-3. Select </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Integrations</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> from the mega menu
-4. Scroll to the search field
-5. Verify the integrations list contains more than one integration
-6. Enter "</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>GitHub</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>" into the search field
-7. Verify the integrations list contains only the "</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>GitHub</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>" integration</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. The </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Developer</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> menu was visible and enabled
-2. The </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Developer</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> mega menu was displayed
-3. The </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Integrations</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> page was opened
-4. The search field was displayed
-5. The integrations list contained more than one integration
-6. "</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>GitHub</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>" was entered into the search field
-7. The integrations list was filtered to display only the "GitHub" integration</t>
-    </r>
-  </si>
-  <si>
     <t>The homepage was opened in a mobile viewport</t>
   </si>
   <si>
@@ -4042,6 +3813,235 @@
       </rPr>
       <t xml:space="preserve"> field was empty
 3. The error notification with the message "Email is required" was displayed</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Verify the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Developers</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> menu is visible and enabled
+2. Click the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Developers</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> menu
+3. Select </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Integrations</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> from the mega menu
+4. Scroll to the search field
+5. Verify the integrations list contains more than one integration
+6. Enter "</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>GitHub</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>" into the search field
+7. Verify the integrations list contains only the "</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>GitHub</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>" integration</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Developers</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> menu was visible and enabled
+2. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Developers</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> mega menu was displayed
+3. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Integrations</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> page was opened
+4. The search field was displayed
+5. The integrations list contained more than one integration
+6. "</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>GitHub</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>" was entered into the search field
+7. The integrations list was filtered to display only the "GitHub" integration</t>
     </r>
   </si>
 </sst>
@@ -4497,7 +4497,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>11</v>
@@ -4545,10 +4545,10 @@
         <v>11</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>6</v>
@@ -4566,10 +4566,10 @@
         <v>28</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>6</v>
@@ -4692,10 +4692,10 @@
         <v>11</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>7</v>
@@ -4710,13 +4710,13 @@
         <v>22</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>6</v>
@@ -4734,10 +4734,10 @@
         <v>11</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>7</v>
@@ -4755,10 +4755,10 @@
         <v>11</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>7</v>
@@ -4770,16 +4770,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>7</v>
@@ -4797,10 +4797,10 @@
         <v>11</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>7</v>
@@ -4818,10 +4818,10 @@
         <v>10</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>7</v>
@@ -4838,10 +4838,10 @@
         <v>11</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>7</v>
@@ -4859,10 +4859,10 @@
         <v>11</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
feat: add content verification tests
</commit_message>
<xml_diff>
--- a/docs/test-cases/TestCases_1.0.xlsx
+++ b/docs/test-cases/TestCases_1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORK\LEARNING\QA Engineer\Internship\5t-wdio-telnyx\docs\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D361D3A-DF76-456B-B8B6-E5B817299178}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16426143-6C01-4899-A06C-C0D643C134E9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1922,396 +1922,6 @@
         <charset val="204"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Pricing</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> menu
-2. Click the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SMS API</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> link from the mega menu
-3. Scroll to </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SENDER Types</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> section
-4. Verify the default tab displays the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Services</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> table with "</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>carrier fee</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">" links
-5. Click on </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>RCS</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> tab
-6. Verify the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Services</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> table is no longer displayed
-7. Verify the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>RCS Rich pricing</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> table heading is displayed</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. The </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Pricing</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> mega menu was displayed
-2. The </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Messaging API</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> page was opened
-3. The </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SENDER Types</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> section was displayed
-4. The "</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>carrier fee</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">" links were displayed in the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Services</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> table
-5. The </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>RCS</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> tab was selected
-6. The </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Services</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> table was no longer displayed
-7. The </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>RCS Rich pricing</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> table heading was displayed</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. Click the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>Resources</t>
     </r>
     <r>
@@ -4042,6 +3652,396 @@
       </rPr>
       <t>" was entered into the search field
 7. The integrations list was filtered to display only the "GitHub" integration</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Click the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Pricing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> menu
+2. Click the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SMS API</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> link from the mega menu
+3. Scroll to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SENDER Types</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> section
+4. Verify the default tab displays the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Services</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> table with "</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>carrier fee</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">" links
+5. Click on </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RCS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tab
+6. Verify the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Services</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> table is no longer displayed
+7. Verify the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RCS Rich pricing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> table is displayed</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Pricing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> mega menu was displayed
+2. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Messaging API</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> page was opened
+3. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SENDER Types</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> section was displayed
+4. The "</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>carrier fee</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">" links were displayed in the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Services</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> table
+5. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RCS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tab was selected
+6. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Services</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> table was no longer displayed
+7. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RCS Rich pricing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> table was displayed</t>
     </r>
   </si>
 </sst>
@@ -4497,7 +4497,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>11</v>
@@ -4545,10 +4545,10 @@
         <v>11</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>6</v>
@@ -4566,10 +4566,10 @@
         <v>28</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>6</v>
@@ -4692,10 +4692,10 @@
         <v>11</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>7</v>
@@ -4713,10 +4713,10 @@
         <v>49</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>6</v>
@@ -4734,10 +4734,10 @@
         <v>11</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>7</v>
@@ -4755,10 +4755,10 @@
         <v>11</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>7</v>
@@ -4770,16 +4770,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>7</v>
@@ -4797,10 +4797,10 @@
         <v>11</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>7</v>
@@ -4818,10 +4818,10 @@
         <v>10</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>7</v>
@@ -4838,10 +4838,10 @@
         <v>11</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>7</v>
@@ -4859,10 +4859,10 @@
         <v>11</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
feat: add dinamic widget tests
</commit_message>
<xml_diff>
--- a/docs/test-cases/TestCases_1.0.xlsx
+++ b/docs/test-cases/TestCases_1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORK\LEARNING\QA Engineer\Internship\5t-wdio-telnyx\docs\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16426143-6C01-4899-A06C-C0D643C134E9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00BEE68D-83CE-4E6F-9529-557EF0F1F47B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2381,61 +2381,6 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> button
-2. Verify the greeting message is displayed
-3. Enter "How can I send a message to the support center?" into the chat input and submit the message
-4. Verify the AI Assistant response is displayed
-5. Click the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Close Widget</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> button</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. Click the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>AI Assistant</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> button
 2. Click the </t>
     </r>
     <r>
@@ -4042,6 +3987,61 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> table was displayed</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Click the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI Assistant</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> button
+2. Verify the greeting message is displayed
+3. Enter "Hello" into the chat input and submit the message
+4. Verify the AI Assistant response is displayed
+5. Click the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Close Widget</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> button</t>
     </r>
   </si>
 </sst>
@@ -4497,7 +4497,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>11</v>
@@ -4545,10 +4545,10 @@
         <v>11</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>67</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>6</v>
@@ -4566,10 +4566,10 @@
         <v>28</v>
       </c>
       <c r="D7" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>68</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>69</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>6</v>
@@ -4692,10 +4692,10 @@
         <v>11</v>
       </c>
       <c r="D13" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>70</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>71</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>7</v>
@@ -4713,10 +4713,10 @@
         <v>49</v>
       </c>
       <c r="D14" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>60</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>61</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>6</v>
@@ -4734,10 +4734,10 @@
         <v>11</v>
       </c>
       <c r="D15" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E15" s="5" t="s">
         <v>72</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>73</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>7</v>
@@ -4758,7 +4758,7 @@
         <v>50</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>7</v>
@@ -4776,10 +4776,10 @@
         <v>11</v>
       </c>
       <c r="D17" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E17" s="5" t="s">
         <v>63</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>64</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>7</v>
@@ -4827,7 +4827,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -4838,7 +4838,7 @@
         <v>11</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>56</v>
@@ -4859,10 +4859,10 @@
         <v>11</v>
       </c>
       <c r="D21" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E21" s="5" t="s">
         <v>58</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>59</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>7</v>

</xml_diff>